<commit_message>
fix: clarify validation results and demo phones
</commit_message>
<xml_diff>
--- a/data/contacts_demo.xlsx
+++ b/data/contacts_demo.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>967770000001</t>
+          <t>+967771234567</t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>967770000002</t>
+          <t>+967731234567</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>967770000003</t>
+          <t>+967711234567</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>967770000004</t>
+          <t>+967701234567</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>967770000005</t>
+          <t>+967781234567</t>
         </is>
       </c>
     </row>

</xml_diff>